<commit_message>
Plano Heinlein: linea de abajo de KGS en bodegas compartidas y linea del casco que se pasaba de la bodega
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/docgen/templates/plano_h5.xlsx
+++ b/app/docgen/templates/plano_h5.xlsx
@@ -706,7 +706,7 @@
       <xdr:row>25</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="866775" cy="38100"/>
+    <xdr:ext cx="749300" cy="38100"/>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
         <xdr:cNvPr id="7" name="Shape 2">
@@ -721,7 +721,7 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="1320165" y="4086225"/>
-          <a:ext cx="866775" cy="38100"/>
+          <a:ext cx="749300" cy="38100"/>
           <a:chOff x="4912613" y="3780000"/>
           <a:chExt cx="866775" cy="0"/>
         </a:xfrm>

</xml_diff>